<commit_message>
add bug reprod instructions
</commit_message>
<xml_diff>
--- a/test_matrix_results/Browser_Test_Matrix_Excel_Orcasound_completed on 7-13-26.xlsx
+++ b/test_matrix_results/Browser_Test_Matrix_Excel_Orcasound_completed on 7-13-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arand\Desktop\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E9F9F80-E368-42B5-AC64-68D9FAECD4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645402B0-27DF-46DF-83A5-AD8560EC94F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="64">
   <si>
     <t>Use ✓ / ✗ / N/A / — to record manual results for each browser and core test case</t>
   </si>
@@ -227,6 +227,33 @@
   </si>
   <si>
     <t>Browser Compatibility Test Matrix completed on 7-13-26</t>
+  </si>
+  <si>
+    <t>Bug Reproduction Instructions.</t>
+  </si>
+  <si>
+    <t>Chrome and Firefox Desktop bug reproduction</t>
+  </si>
+  <si>
+    <t>Android Chrome and Firefox bug reproduction</t>
+  </si>
+  <si>
+    <t>Safari Desktop bug reproduction</t>
+  </si>
+  <si>
+    <t>To reproduce the bugs listed for Safari, use browser stack live and connect to an Apple desktop device or use a personal device if the tester uses an Apple Desktop computer. To reproduce the bugs for Safari Desktop, simply use the same process that is used for Chrome and Firefox Desktop bug reproduction. Navigate to the pages listed and inspect the pages. To trigger error build on About Us, same process as with windows, simply navigate using the nav bar link and the build error is triggered.</t>
+  </si>
+  <si>
+    <t>IOS Safari bug reproduction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To reproduce the bugs listed for the Chrome and Firefox Desktop simply navigate to home, get involved, learn, hacker hall of fame, call catalog, and support me (donate) and inspect by pressing F12 or right clicking and pressing inspect in the tab menu. They'll be listed in the console. The bugs happen automatically after mounting, there isn't a specific action or event that triggers them other than navigating to the page. For the error that occurs on About Us, same thing, simply navigate to the page via nav bar and the error occurs.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">For reproduction of the bugs on Android, use Browser Stack or can use the mobile feature on dev tools for each browser and pick an Android device. Since all the bugs list for Desktop are the same here, reproducing them is exactly the same process. Simply navigate to each page: home, get involved, learn, hacker hall of fame, and call catalog. Right click and inspect on each page. Now, I didn't list the donate page for navigation and inspection because that's one of the errors for mobile. On Tablet and Android devices when you click on the three horizontal bars in the top right of the nav bar, hamburger symbol, you'll see all the links for the other pages except the donate page link. It's not there when using the app on Android or Tablet. For the About Us page, simply navigate by clicking on the link to the page in the nav bar via the hamburger symbol and the build error will occur. </t>
+  </si>
+  <si>
+    <t>Bug reproduction for Iphone and Ipad is the same as Android and Tablet. Use browser stack or personal devices and navigate to the pages listed in the Android test. Right click and inspect each page.  The warnings and errors listed will appear in the console. The donate page link does not appear when the hamburger symbol in the nav bar is clicked. The About Us page error happens by simply clicking on the link to the page in the nav bar after clicking the hamburger symbol.</t>
   </si>
 </sst>
 </file>
@@ -311,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -344,6 +371,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -556,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1041,11 +1074,215 @@
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
     </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="15"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="15"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="15"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="15"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="15"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="15"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="15"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="15"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="15"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="15"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="15"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="15"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="15"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="12">
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A60:C65"/>
+    <mergeCell ref="A26:C34"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A38:C44"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A48:C55"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:C25"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:I14">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>